<commit_message>
fixes not completed and added step 9 & 10
</commit_message>
<xml_diff>
--- a/STEP2_ML/Step7_ML_Baseline_Regression.xlsx
+++ b/STEP2_ML/Step7_ML_Baseline_Regression.xlsx
@@ -490,7 +490,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-26 16:47:18</t>
+          <t>2026-10-02 20:34:54</t>
         </is>
       </c>
     </row>
@@ -761,7 +761,7 @@
         <v>0.934595006210568</v>
       </c>
       <c r="D2" t="n">
-        <v>0.04789873615059224</v>
+        <v>0.04789873615059226</v>
       </c>
       <c r="E2" t="n">
         <v>0.05773522570429511</v>
@@ -770,16 +770,16 @@
         <v>0.02632622707999459</v>
       </c>
       <c r="G2" t="n">
-        <v>0.03880812837383148</v>
+        <v>0.0388081283738315</v>
       </c>
       <c r="H2" t="n">
-        <v>0.01378196536571906</v>
+        <v>0.01378196536571907</v>
       </c>
       <c r="I2" t="n">
-        <v>30.61306122687439</v>
+        <v>30.6130612268744</v>
       </c>
       <c r="J2" t="n">
-        <v>43.29885535490735</v>
+        <v>43.29885535490737</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
@@ -800,7 +800,7 @@
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>2.22</v>
+        <v>1.85</v>
       </c>
       <c r="R2" t="n">
         <v>1</v>
@@ -881,22 +881,22 @@
         <v>0.9086835175888824</v>
       </c>
       <c r="D4" t="n">
-        <v>0.07157281593152007</v>
+        <v>0.07157281593152004</v>
       </c>
       <c r="E4" t="n">
-        <v>0.06743308713174541</v>
+        <v>0.06743308713174538</v>
       </c>
       <c r="F4" t="n">
-        <v>0.02975830046271981</v>
+        <v>0.02975830046271982</v>
       </c>
       <c r="G4" t="n">
-        <v>0.04687164893782945</v>
+        <v>0.04687164893782944</v>
       </c>
       <c r="H4" t="n">
-        <v>0.01565195724785954</v>
+        <v>0.01565195724785955</v>
       </c>
       <c r="I4" t="n">
-        <v>37.38542691849484</v>
+        <v>37.38542691849482</v>
       </c>
       <c r="J4" t="n">
         <v>44.10015139623641</v>
@@ -908,10 +908,10 @@
         <v>0.9205465657834363</v>
       </c>
       <c r="M4" t="n">
-        <v>0.07146766866324994</v>
+        <v>0.07146766866324993</v>
       </c>
       <c r="N4" t="n">
-        <v>0.04582092310124124</v>
+        <v>0.04582092310124122</v>
       </c>
       <c r="O4" t="n">
         <v>37.12762240188454</v>
@@ -920,7 +920,7 @@
         <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>2.91</v>
+        <v>2.54</v>
       </c>
       <c r="R4" t="n">
         <v>3</v>
@@ -980,7 +980,7 @@
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>1.17</v>
+        <v>0.89</v>
       </c>
       <c r="R5" t="n">
         <v>4</v>
@@ -1100,7 +1100,7 @@
         <v>2</v>
       </c>
       <c r="Q7" t="n">
-        <v>1.88</v>
+        <v>1.69</v>
       </c>
       <c r="R7" t="n">
         <v>6</v>
@@ -1160,7 +1160,7 @@
         <v>6</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.8</v>
+        <v>0.45</v>
       </c>
       <c r="R8" t="n">
         <v>7</v>
@@ -1220,7 +1220,7 @@
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>1.55</v>
+        <v>1.69</v>
       </c>
       <c r="R9" t="n">
         <v>1</v>
@@ -1280,7 +1280,7 @@
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="R10" t="n">
         <v>2</v>
@@ -1340,7 +1340,7 @@
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.66</v>
+        <v>0.86</v>
       </c>
       <c r="R11" t="n">
         <v>3</v>
@@ -1400,7 +1400,7 @@
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>1.84</v>
+        <v>1.97</v>
       </c>
       <c r="R12" t="n">
         <v>4</v>
@@ -1421,25 +1421,25 @@
         <v>0.9374010843496684</v>
       </c>
       <c r="D13" t="n">
-        <v>0.05379048162956031</v>
+        <v>0.05379048162956027</v>
       </c>
       <c r="E13" t="n">
-        <v>0.2165773128946292</v>
+        <v>0.2165773128946291</v>
       </c>
       <c r="F13" t="n">
-        <v>0.107498551549062</v>
+        <v>0.1074985515490619</v>
       </c>
       <c r="G13" t="n">
-        <v>0.1479875453559632</v>
+        <v>0.1479875453559631</v>
       </c>
       <c r="H13" t="n">
-        <v>0.06153312495000573</v>
+        <v>0.06153312495000569</v>
       </c>
       <c r="I13" t="n">
-        <v>8.528605207321654</v>
+        <v>8.528605207321652</v>
       </c>
       <c r="J13" t="n">
-        <v>5.394008431998433</v>
+        <v>5.39400843199843</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
@@ -1460,7 +1460,7 @@
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>2.55</v>
+        <v>2.57</v>
       </c>
       <c r="R13" t="n">
         <v>5</v>
@@ -1481,7 +1481,7 @@
         <v>0.9237199152618111</v>
       </c>
       <c r="D14" t="n">
-        <v>0.09033705819320621</v>
+        <v>0.0903370581932061</v>
       </c>
       <c r="E14" t="n">
         <v>0.2252485299846607</v>
@@ -1499,7 +1499,7 @@
         <v>8.838734822898127</v>
       </c>
       <c r="J14" t="n">
-        <v>6.583023766051228</v>
+        <v>6.583023766051226</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
@@ -1508,19 +1508,19 @@
         <v>0.929186656094704</v>
       </c>
       <c r="M14" t="n">
-        <v>0.2547375872727886</v>
+        <v>0.2547375872727887</v>
       </c>
       <c r="N14" t="n">
         <v>0.1357433249875997</v>
       </c>
       <c r="O14" t="n">
-        <v>8.637390708234369</v>
+        <v>8.637390708234371</v>
       </c>
       <c r="P14" t="n">
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>1.89</v>
+        <v>1.93</v>
       </c>
       <c r="R14" t="n">
         <v>6</v>
@@ -1601,25 +1601,25 @@
         <v>0.9644925796153505</v>
       </c>
       <c r="D16" t="n">
-        <v>0.01851395006701762</v>
+        <v>0.01851395006701763</v>
       </c>
       <c r="E16" t="n">
         <v>0.01698790673322198</v>
       </c>
       <c r="F16" t="n">
-        <v>0.005677820350172568</v>
+        <v>0.005677820350172569</v>
       </c>
       <c r="G16" t="n">
         <v>0.01255353215110581</v>
       </c>
       <c r="H16" t="n">
-        <v>0.003854235163110614</v>
+        <v>0.003854235163110611</v>
       </c>
       <c r="I16" t="n">
         <v>11.56299647859421</v>
       </c>
       <c r="J16" t="n">
-        <v>5.935209141622209</v>
+        <v>5.935209141622207</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
@@ -1628,7 +1628,7 @@
         <v>0.9691747585733861</v>
       </c>
       <c r="M16" t="n">
-        <v>0.01693254348005207</v>
+        <v>0.01693254348005208</v>
       </c>
       <c r="N16" t="n">
         <v>0.01226590158283614</v>
@@ -1640,7 +1640,7 @@
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.86</v>
+        <v>1.88</v>
       </c>
       <c r="R16" t="n">
         <v>1</v>
@@ -1661,25 +1661,25 @@
         <v>0.9574844716642613</v>
       </c>
       <c r="D17" t="n">
-        <v>0.0231294604355229</v>
+        <v>0.02312946043552292</v>
       </c>
       <c r="E17" t="n">
-        <v>0.01841844557136577</v>
+        <v>0.01841844557136578</v>
       </c>
       <c r="F17" t="n">
-        <v>0.004342099208328032</v>
+        <v>0.004342099208328037</v>
       </c>
       <c r="G17" t="n">
         <v>0.01451788011675299</v>
       </c>
       <c r="H17" t="n">
-        <v>0.003499896687615539</v>
+        <v>0.003499896687615544</v>
       </c>
       <c r="I17" t="n">
         <v>11.62987978932676</v>
       </c>
       <c r="J17" t="n">
-        <v>4.950195591049303</v>
+        <v>4.950195591049299</v>
       </c>
       <c r="K17" t="n">
         <v>0</v>
@@ -1691,7 +1691,7 @@
         <v>0.01803234270031003</v>
       </c>
       <c r="N17" t="n">
-        <v>0.01401492211374606</v>
+        <v>0.01401492211374607</v>
       </c>
       <c r="O17" t="n">
         <v>11.22639972317902</v>
@@ -1700,7 +1700,7 @@
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>2.52</v>
+        <v>2.58</v>
       </c>
       <c r="R17" t="n">
         <v>2</v>
@@ -1820,7 +1820,7 @@
         <v>0</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.57</v>
+        <v>0.68</v>
       </c>
       <c r="R19" t="n">
         <v>4</v>
@@ -1940,7 +1940,7 @@
         <v>3</v>
       </c>
       <c r="Q21" t="n">
-        <v>1.66</v>
+        <v>1.68</v>
       </c>
       <c r="R21" t="n">
         <v>6</v>
@@ -2000,7 +2000,7 @@
         <v>2</v>
       </c>
       <c r="Q22" t="n">
-        <v>0.25</v>
+        <v>0.23</v>
       </c>
       <c r="R22" t="n">
         <v>7</v>
@@ -2122,22 +2122,22 @@
         <v>0.9086835175888824</v>
       </c>
       <c r="D2" t="n">
-        <v>0.07157281593152007</v>
+        <v>0.07157281593152004</v>
       </c>
       <c r="E2" t="n">
-        <v>0.06743308713174541</v>
+        <v>0.06743308713174538</v>
       </c>
       <c r="F2" t="n">
-        <v>0.02975830046271981</v>
+        <v>0.02975830046271982</v>
       </c>
       <c r="G2" t="n">
-        <v>0.04687164893782945</v>
+        <v>0.04687164893782944</v>
       </c>
       <c r="H2" t="n">
-        <v>0.01565195724785954</v>
+        <v>0.01565195724785955</v>
       </c>
       <c r="I2" t="n">
-        <v>37.38542691849484</v>
+        <v>37.38542691849482</v>
       </c>
       <c r="J2" t="n">
         <v>44.10015139623641</v>
@@ -2149,10 +2149,10 @@
         <v>0.9205465657834363</v>
       </c>
       <c r="M2" t="n">
-        <v>0.07146766866324994</v>
+        <v>0.07146766866324993</v>
       </c>
       <c r="N2" t="n">
-        <v>0.04582092310124124</v>
+        <v>0.04582092310124122</v>
       </c>
       <c r="O2" t="n">
         <v>37.12762240188454</v>
@@ -2161,7 +2161,7 @@
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>2.91</v>
+        <v>2.54</v>
       </c>
     </row>
     <row r="3">
@@ -2179,7 +2179,7 @@
         <v>0.934595006210568</v>
       </c>
       <c r="D3" t="n">
-        <v>0.04789873615059224</v>
+        <v>0.04789873615059226</v>
       </c>
       <c r="E3" t="n">
         <v>0.05773522570429511</v>
@@ -2188,16 +2188,16 @@
         <v>0.02632622707999459</v>
       </c>
       <c r="G3" t="n">
-        <v>0.03880812837383148</v>
+        <v>0.0388081283738315</v>
       </c>
       <c r="H3" t="n">
-        <v>0.01378196536571906</v>
+        <v>0.01378196536571907</v>
       </c>
       <c r="I3" t="n">
-        <v>30.61306122687439</v>
+        <v>30.6130612268744</v>
       </c>
       <c r="J3" t="n">
-        <v>43.29885535490735</v>
+        <v>43.29885535490737</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
@@ -2218,7 +2218,7 @@
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>2.22</v>
+        <v>1.85</v>
       </c>
     </row>
     <row r="4">
@@ -2275,7 +2275,7 @@
         <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>1.17</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="5">
@@ -2446,7 +2446,7 @@
         <v>6</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.8</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="8">
@@ -2503,7 +2503,7 @@
         <v>2</v>
       </c>
       <c r="Q8" t="n">
-        <v>1.88</v>
+        <v>1.69</v>
       </c>
     </row>
     <row r="9">
@@ -2521,25 +2521,25 @@
         <v>0.9374010843496684</v>
       </c>
       <c r="D9" t="n">
-        <v>0.05379048162956031</v>
+        <v>0.05379048162956027</v>
       </c>
       <c r="E9" t="n">
-        <v>0.2165773128946292</v>
+        <v>0.2165773128946291</v>
       </c>
       <c r="F9" t="n">
-        <v>0.107498551549062</v>
+        <v>0.1074985515490619</v>
       </c>
       <c r="G9" t="n">
-        <v>0.1479875453559632</v>
+        <v>0.1479875453559631</v>
       </c>
       <c r="H9" t="n">
-        <v>0.06153312495000573</v>
+        <v>0.06153312495000569</v>
       </c>
       <c r="I9" t="n">
-        <v>8.528605207321654</v>
+        <v>8.528605207321652</v>
       </c>
       <c r="J9" t="n">
-        <v>5.394008431998433</v>
+        <v>5.39400843199843</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
@@ -2560,7 +2560,7 @@
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>2.55</v>
+        <v>2.57</v>
       </c>
     </row>
     <row r="10">
@@ -2578,7 +2578,7 @@
         <v>0.9237199152618111</v>
       </c>
       <c r="D10" t="n">
-        <v>0.09033705819320621</v>
+        <v>0.0903370581932061</v>
       </c>
       <c r="E10" t="n">
         <v>0.2252485299846607</v>
@@ -2596,7 +2596,7 @@
         <v>8.838734822898127</v>
       </c>
       <c r="J10" t="n">
-        <v>6.583023766051228</v>
+        <v>6.583023766051226</v>
       </c>
       <c r="K10" t="n">
         <v>0</v>
@@ -2605,19 +2605,19 @@
         <v>0.929186656094704</v>
       </c>
       <c r="M10" t="n">
-        <v>0.2547375872727886</v>
+        <v>0.2547375872727887</v>
       </c>
       <c r="N10" t="n">
         <v>0.1357433249875997</v>
       </c>
       <c r="O10" t="n">
-        <v>8.637390708234369</v>
+        <v>8.637390708234371</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>1.89</v>
+        <v>1.93</v>
       </c>
     </row>
     <row r="11">
@@ -2674,7 +2674,7 @@
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.66</v>
+        <v>0.86</v>
       </c>
     </row>
     <row r="12">
@@ -2731,7 +2731,7 @@
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="13">
@@ -2845,7 +2845,7 @@
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>1.84</v>
+        <v>1.97</v>
       </c>
     </row>
     <row r="15">
@@ -2902,7 +2902,7 @@
         <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.55</v>
+        <v>1.69</v>
       </c>
     </row>
     <row r="16">
@@ -2920,25 +2920,25 @@
         <v>0.9574844716642613</v>
       </c>
       <c r="D16" t="n">
-        <v>0.0231294604355229</v>
+        <v>0.02312946043552292</v>
       </c>
       <c r="E16" t="n">
-        <v>0.01841844557136577</v>
+        <v>0.01841844557136578</v>
       </c>
       <c r="F16" t="n">
-        <v>0.004342099208328032</v>
+        <v>0.004342099208328037</v>
       </c>
       <c r="G16" t="n">
         <v>0.01451788011675299</v>
       </c>
       <c r="H16" t="n">
-        <v>0.003499896687615539</v>
+        <v>0.003499896687615544</v>
       </c>
       <c r="I16" t="n">
         <v>11.62987978932676</v>
       </c>
       <c r="J16" t="n">
-        <v>4.950195591049303</v>
+        <v>4.950195591049299</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
@@ -2950,7 +2950,7 @@
         <v>0.01803234270031003</v>
       </c>
       <c r="N16" t="n">
-        <v>0.01401492211374606</v>
+        <v>0.01401492211374607</v>
       </c>
       <c r="O16" t="n">
         <v>11.22639972317902</v>
@@ -2959,7 +2959,7 @@
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>2.52</v>
+        <v>2.58</v>
       </c>
     </row>
     <row r="17">
@@ -2977,25 +2977,25 @@
         <v>0.9644925796153505</v>
       </c>
       <c r="D17" t="n">
-        <v>0.01851395006701762</v>
+        <v>0.01851395006701763</v>
       </c>
       <c r="E17" t="n">
         <v>0.01698790673322198</v>
       </c>
       <c r="F17" t="n">
-        <v>0.005677820350172568</v>
+        <v>0.005677820350172569</v>
       </c>
       <c r="G17" t="n">
         <v>0.01255353215110581</v>
       </c>
       <c r="H17" t="n">
-        <v>0.003854235163110614</v>
+        <v>0.003854235163110611</v>
       </c>
       <c r="I17" t="n">
         <v>11.56299647859421</v>
       </c>
       <c r="J17" t="n">
-        <v>5.935209141622209</v>
+        <v>5.935209141622207</v>
       </c>
       <c r="K17" t="n">
         <v>0</v>
@@ -3004,7 +3004,7 @@
         <v>0.9691747585733861</v>
       </c>
       <c r="M17" t="n">
-        <v>0.01693254348005207</v>
+        <v>0.01693254348005208</v>
       </c>
       <c r="N17" t="n">
         <v>0.01226590158283614</v>
@@ -3016,7 +3016,7 @@
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>1.86</v>
+        <v>1.88</v>
       </c>
     </row>
     <row r="18">
@@ -3073,7 +3073,7 @@
         <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.57</v>
+        <v>0.68</v>
       </c>
     </row>
     <row r="19">
@@ -3244,7 +3244,7 @@
         <v>2</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.25</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="22">
@@ -3301,7 +3301,7 @@
         <v>3</v>
       </c>
       <c r="Q22" t="n">
-        <v>1.66</v>
+        <v>1.68</v>
       </c>
     </row>
   </sheetData>
@@ -3388,10 +3388,10 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>0.7729056664181835</v>
+        <v>0.7729056664181837</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1023759795928143</v>
+        <v>0.1023759795928142</v>
       </c>
       <c r="G2" t="n">
         <v>0.06699161548691163</v>
@@ -3424,13 +3424,13 @@
         <v>2</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9879939754543905</v>
+        <v>0.9879939754543904</v>
       </c>
       <c r="F3" t="n">
-        <v>0.02898524985974773</v>
+        <v>0.02898524985974774</v>
       </c>
       <c r="G3" t="n">
-        <v>0.02246299386743996</v>
+        <v>0.02246299386743993</v>
       </c>
       <c r="H3" t="n">
         <v>15.47624150976244</v>
@@ -3460,16 +3460,16 @@
         <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9487139417988143</v>
+        <v>0.9487139417988144</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0427611375028271</v>
+        <v>0.04276113750282704</v>
       </c>
       <c r="G4" t="n">
-        <v>0.03505068827182459</v>
+        <v>0.03505068827182451</v>
       </c>
       <c r="H4" t="n">
-        <v>6.674419909908141</v>
+        <v>6.67441990990813</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
@@ -3496,13 +3496,13 @@
         <v>4</v>
       </c>
       <c r="E5" t="n">
-        <v>0.8506904686185527</v>
+        <v>0.8506904686185526</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1298798554352994</v>
+        <v>0.1298798554352995</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0758159436458514</v>
+        <v>0.07581594364585145</v>
       </c>
       <c r="H5" t="n">
         <v>162.6883983244414</v>
@@ -3532,16 +3532,16 @@
         <v>5</v>
       </c>
       <c r="E6" t="n">
-        <v>0.9554153769739882</v>
+        <v>0.9554153769739883</v>
       </c>
       <c r="F6" t="n">
-        <v>0.04652566682652855</v>
+        <v>0.04652566682652853</v>
       </c>
       <c r="G6" t="n">
-        <v>0.03443792986443413</v>
+        <v>0.03443792986443405</v>
       </c>
       <c r="H6" t="n">
-        <v>6.719143977604316</v>
+        <v>6.719143977604306</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -3571,7 +3571,7 @@
         <v>0.960679300842899</v>
       </c>
       <c r="F7" t="n">
-        <v>0.04585896217711714</v>
+        <v>0.04585896217711711</v>
       </c>
       <c r="G7" t="n">
         <v>0.03824346555197693</v>
@@ -3604,16 +3604,16 @@
         <v>2</v>
       </c>
       <c r="E8" t="n">
-        <v>0.7928949942950517</v>
+        <v>0.7928949942950518</v>
       </c>
       <c r="F8" t="n">
         <v>0.1022127662201955</v>
       </c>
       <c r="G8" t="n">
-        <v>0.06396053949446141</v>
+        <v>0.06396053949446134</v>
       </c>
       <c r="H8" t="n">
-        <v>79.10616395599142</v>
+        <v>79.10616395599135</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
@@ -3646,7 +3646,7 @@
         <v>0.07536887739731302</v>
       </c>
       <c r="G9" t="n">
-        <v>0.05469368741172091</v>
+        <v>0.05469368741172092</v>
       </c>
       <c r="H9" t="n">
         <v>34.47562124565165</v>
@@ -3676,16 +3676,16 @@
         <v>4</v>
       </c>
       <c r="E10" t="n">
-        <v>0.9611278560795318</v>
+        <v>0.9611278560795319</v>
       </c>
       <c r="F10" t="n">
-        <v>0.05778224191101445</v>
+        <v>0.05778224191101443</v>
       </c>
       <c r="G10" t="n">
-        <v>0.04398853709277636</v>
+        <v>0.04398853709277639</v>
       </c>
       <c r="H10" t="n">
-        <v>31.09237382655139</v>
+        <v>31.09237382655137</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -3715,13 +3715,13 @@
         <v>0.9569499896821947</v>
       </c>
       <c r="F11" t="n">
-        <v>0.04103456627056729</v>
+        <v>0.04103456627056732</v>
       </c>
       <c r="G11" t="n">
-        <v>0.03336658306607083</v>
+        <v>0.03336658306607088</v>
       </c>
       <c r="H11" t="n">
-        <v>6.863525608826563</v>
+        <v>6.863525608826572</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
@@ -3751,13 +3751,13 @@
         <v>0.9807244391706221</v>
       </c>
       <c r="F12" t="n">
-        <v>0.03354751798682628</v>
+        <v>0.0335475179868262</v>
       </c>
       <c r="G12" t="n">
-        <v>0.02635031425088559</v>
+        <v>0.02635031425088553</v>
       </c>
       <c r="H12" t="n">
-        <v>6.446016562673204</v>
+        <v>6.446016562673197</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
@@ -3784,16 +3784,16 @@
         <v>2</v>
       </c>
       <c r="E13" t="n">
-        <v>0.9358009787136877</v>
+        <v>0.9358009787136878</v>
       </c>
       <c r="F13" t="n">
-        <v>0.07895166030474536</v>
+        <v>0.07895166030474531</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0587339364665631</v>
+        <v>0.05873393646656305</v>
       </c>
       <c r="H13" t="n">
-        <v>82.07642288964728</v>
+        <v>82.07642288964726</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
@@ -3829,7 +3829,7 @@
         <v>0.06367670311210774</v>
       </c>
       <c r="H14" t="n">
-        <v>87.48901227121679</v>
+        <v>87.48901227121681</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -3856,13 +3856,13 @@
         <v>4</v>
       </c>
       <c r="E15" t="n">
-        <v>0.9568678387485584</v>
+        <v>0.9568678387485585</v>
       </c>
       <c r="F15" t="n">
-        <v>0.04920399255807834</v>
+        <v>0.04920399255807827</v>
       </c>
       <c r="G15" t="n">
-        <v>0.03797015057596403</v>
+        <v>0.037970150575964</v>
       </c>
       <c r="H15" t="n">
         <v>11.63846683941818</v>
@@ -3892,16 +3892,16 @@
         <v>5</v>
       </c>
       <c r="E16" t="n">
-        <v>0.8269045776050911</v>
+        <v>0.826904577605091</v>
       </c>
       <c r="F16" t="n">
-        <v>0.07104761047268245</v>
+        <v>0.07104761047268246</v>
       </c>
       <c r="G16" t="n">
-        <v>0.0473316459084533</v>
+        <v>0.04733164590845334</v>
       </c>
       <c r="H16" t="n">
-        <v>8.873495203991801</v>
+        <v>8.873495203991805</v>
       </c>
       <c r="I16" t="n">
         <v>0</v>
@@ -3934,7 +3934,7 @@
         <v>0.07819767631510688</v>
       </c>
       <c r="G17" t="n">
-        <v>0.0545439026221111</v>
+        <v>0.05454390262211114</v>
       </c>
       <c r="H17" t="n">
         <v>11.94509832504976</v>
@@ -3970,10 +3970,10 @@
         <v>0.01956079887487927</v>
       </c>
       <c r="G18" t="n">
-        <v>0.01700559533123231</v>
+        <v>0.01700559533123229</v>
       </c>
       <c r="H18" t="n">
-        <v>4.820017045401428</v>
+        <v>4.820017045401424</v>
       </c>
       <c r="I18" t="n">
         <v>0</v>
@@ -4003,10 +4003,10 @@
         <v>0.9770438340858895</v>
       </c>
       <c r="F19" t="n">
-        <v>0.02860877528881058</v>
+        <v>0.0286087752888106</v>
       </c>
       <c r="G19" t="n">
-        <v>0.02500632246787091</v>
+        <v>0.02500632246787092</v>
       </c>
       <c r="H19" t="n">
         <v>4.034092829750668</v>
@@ -4036,13 +4036,13 @@
         <v>4</v>
       </c>
       <c r="E20" t="n">
-        <v>0.857507600473096</v>
+        <v>0.8575076004730959</v>
       </c>
       <c r="F20" t="n">
-        <v>0.1268802075268829</v>
+        <v>0.126880207526883</v>
       </c>
       <c r="G20" t="n">
-        <v>0.07149343308632337</v>
+        <v>0.0714934330863234</v>
       </c>
       <c r="H20" t="n">
         <v>169.0888449669183</v>
@@ -4072,16 +4072,16 @@
         <v>5</v>
       </c>
       <c r="E21" t="n">
-        <v>0.9466057259767559</v>
+        <v>0.9466057259767557</v>
       </c>
       <c r="F21" t="n">
-        <v>0.05091519364832107</v>
+        <v>0.05091519364832112</v>
       </c>
       <c r="G21" t="n">
-        <v>0.03446981065470142</v>
+        <v>0.03446981065470146</v>
       </c>
       <c r="H21" t="n">
-        <v>7.265339339639556</v>
+        <v>7.265339339639562</v>
       </c>
       <c r="I21" t="n">
         <v>0</v>
@@ -4111,13 +4111,13 @@
         <v>0.9642850211250396</v>
       </c>
       <c r="F22" t="n">
-        <v>0.04370577294260217</v>
+        <v>0.04370577294260219</v>
       </c>
       <c r="G22" t="n">
-        <v>0.03435584038061213</v>
+        <v>0.03435584038061223</v>
       </c>
       <c r="H22" t="n">
-        <v>8.740638404883152</v>
+        <v>8.740638404883159</v>
       </c>
       <c r="I22" t="n">
         <v>0</v>
@@ -4147,13 +4147,13 @@
         <v>0.902470815172052</v>
       </c>
       <c r="F23" t="n">
-        <v>0.07014183786378553</v>
+        <v>0.07014183786378551</v>
       </c>
       <c r="G23" t="n">
-        <v>0.03980077470066901</v>
+        <v>0.03980077470066893</v>
       </c>
       <c r="H23" t="n">
-        <v>56.29859274977699</v>
+        <v>56.29859274977698</v>
       </c>
       <c r="I23" t="n">
         <v>0</v>
@@ -4186,7 +4186,7 @@
         <v>0.07787012532891494</v>
       </c>
       <c r="G24" t="n">
-        <v>0.05197189259621079</v>
+        <v>0.05197189259621076</v>
       </c>
       <c r="H24" t="n">
         <v>13.61721683403763</v>
@@ -4219,13 +4219,13 @@
         <v>0.9816164863215283</v>
       </c>
       <c r="F25" t="n">
-        <v>0.03973648085434249</v>
+        <v>0.03973648085434247</v>
       </c>
       <c r="G25" t="n">
-        <v>0.02444527328754498</v>
+        <v>0.02444527328754494</v>
       </c>
       <c r="H25" t="n">
-        <v>12.41983997497822</v>
+        <v>12.41983997497821</v>
       </c>
       <c r="I25" t="n">
         <v>0</v>
@@ -4252,13 +4252,13 @@
         <v>5</v>
       </c>
       <c r="E26" t="n">
-        <v>0.9792628787589855</v>
+        <v>0.9792628787589857</v>
       </c>
       <c r="F26" t="n">
-        <v>0.02847983381733089</v>
+        <v>0.02847983381733087</v>
       </c>
       <c r="G26" t="n">
-        <v>0.02631878299210461</v>
+        <v>0.0263187829921046</v>
       </c>
       <c r="H26" t="n">
         <v>4.480580222169713</v>
@@ -4288,16 +4288,16 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>0.9716434954073986</v>
+        <v>0.9716434954073985</v>
       </c>
       <c r="F27" t="n">
-        <v>0.04068958223374503</v>
+        <v>0.04068958223374507</v>
       </c>
       <c r="G27" t="n">
-        <v>0.03127875377605191</v>
+        <v>0.03127875377605194</v>
       </c>
       <c r="H27" t="n">
-        <v>8.774334298332771</v>
+        <v>8.774334298332779</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
@@ -4330,7 +4330,7 @@
         <v>0.06867465680192657</v>
       </c>
       <c r="G28" t="n">
-        <v>0.04568603556217303</v>
+        <v>0.04568603556217304</v>
       </c>
       <c r="H28" t="n">
         <v>75.54392472941632</v>
@@ -4366,10 +4366,10 @@
         <v>0.07507078325521613</v>
       </c>
       <c r="G29" t="n">
-        <v>0.0483951418536341</v>
+        <v>0.04839514185363415</v>
       </c>
       <c r="H29" t="n">
-        <v>61.13146848327706</v>
+        <v>61.13146848327708</v>
       </c>
       <c r="I29" t="n">
         <v>0</v>
@@ -4402,10 +4402,10 @@
         <v>0.0488648260322033</v>
       </c>
       <c r="G30" t="n">
-        <v>0.03173897426064125</v>
+        <v>0.03173897426064121</v>
       </c>
       <c r="H30" t="n">
-        <v>12.15646309706664</v>
+        <v>12.15646309706663</v>
       </c>
       <c r="I30" t="n">
         <v>0</v>
@@ -4435,13 +4435,13 @@
         <v>0.8384757067161029</v>
       </c>
       <c r="F31" t="n">
-        <v>0.06863183478035888</v>
+        <v>0.06863183478035886</v>
       </c>
       <c r="G31" t="n">
-        <v>0.04561139203559143</v>
+        <v>0.04561139203559147</v>
       </c>
       <c r="H31" t="n">
-        <v>8.879467102417655</v>
+        <v>8.879467102417658</v>
       </c>
       <c r="I31" t="n">
         <v>0</v>
@@ -7171,13 +7171,13 @@
         <v>0.9905583893940074</v>
       </c>
       <c r="F107" t="n">
-        <v>0.09717281889816075</v>
+        <v>0.09717281889816073</v>
       </c>
       <c r="G107" t="n">
-        <v>0.07758712662434744</v>
+        <v>0.07758712662434743</v>
       </c>
       <c r="H107" t="n">
-        <v>4.679577714293914</v>
+        <v>4.679577714293915</v>
       </c>
       <c r="I107" t="n">
         <v>0</v>
@@ -7204,16 +7204,16 @@
         <v>2</v>
       </c>
       <c r="E108" t="n">
-        <v>0.9356688382725566</v>
+        <v>0.9356688382725568</v>
       </c>
       <c r="F108" t="n">
-        <v>0.2282317971578707</v>
+        <v>0.2282317971578705</v>
       </c>
       <c r="G108" t="n">
-        <v>0.1523089435791102</v>
+        <v>0.15230894357911</v>
       </c>
       <c r="H108" t="n">
-        <v>8.327269032201654</v>
+        <v>8.327269032201652</v>
       </c>
       <c r="I108" t="n">
         <v>0</v>
@@ -7246,10 +7246,10 @@
         <v>0.1712916390350722</v>
       </c>
       <c r="G109" t="n">
-        <v>0.1029406064662091</v>
+        <v>0.1029406064662092</v>
       </c>
       <c r="H109" t="n">
-        <v>3.656360257285203</v>
+        <v>3.656360257285206</v>
       </c>
       <c r="I109" t="n">
         <v>0</v>
@@ -7276,16 +7276,16 @@
         <v>4</v>
       </c>
       <c r="E110" t="n">
-        <v>0.7998044285801578</v>
+        <v>0.799804428580158</v>
       </c>
       <c r="F110" t="n">
-        <v>0.4423680767250065</v>
+        <v>0.4423680767250062</v>
       </c>
       <c r="G110" t="n">
-        <v>0.2355401245133124</v>
+        <v>0.2355401245133122</v>
       </c>
       <c r="H110" t="n">
-        <v>19.46053373416628</v>
+        <v>19.46053373416626</v>
       </c>
       <c r="I110" t="n">
         <v>0</v>
@@ -7315,13 +7315,13 @@
         <v>0.9481803733836008</v>
       </c>
       <c r="F111" t="n">
-        <v>0.1776688587531539</v>
+        <v>0.1776688587531538</v>
       </c>
       <c r="G111" t="n">
-        <v>0.1317039491753529</v>
+        <v>0.1317039491753528</v>
       </c>
       <c r="H111" t="n">
-        <v>5.811078989822661</v>
+        <v>5.811078989822656</v>
       </c>
       <c r="I111" t="n">
         <v>0</v>
@@ -7354,10 +7354,10 @@
         <v>0.1086025120422326</v>
       </c>
       <c r="G112" t="n">
-        <v>0.07974809654720127</v>
+        <v>0.07974809654720137</v>
       </c>
       <c r="H112" t="n">
-        <v>3.000676849170385</v>
+        <v>3.00067684917039</v>
       </c>
       <c r="I112" t="n">
         <v>0</v>
@@ -7387,13 +7387,13 @@
         <v>0.9640569438548063</v>
       </c>
       <c r="F113" t="n">
-        <v>0.2043583234897562</v>
+        <v>0.2043583234897564</v>
       </c>
       <c r="G113" t="n">
-        <v>0.1481906326444815</v>
+        <v>0.1481906326444817</v>
       </c>
       <c r="H113" t="n">
-        <v>7.092790110053484</v>
+        <v>7.09279011005349</v>
       </c>
       <c r="I113" t="n">
         <v>0</v>
@@ -7420,10 +7420,10 @@
         <v>3</v>
       </c>
       <c r="E114" t="n">
-        <v>0.8972098979658163</v>
+        <v>0.8972098979658162</v>
       </c>
       <c r="F114" t="n">
-        <v>0.2931537311417737</v>
+        <v>0.2931537311417738</v>
       </c>
       <c r="G114" t="n">
         <v>0.1945777266790306</v>
@@ -7459,13 +7459,13 @@
         <v>0.8598475723702497</v>
       </c>
       <c r="F115" t="n">
-        <v>0.316393958241846</v>
+        <v>0.3163939582418459</v>
       </c>
       <c r="G115" t="n">
-        <v>0.2287938424346994</v>
+        <v>0.2287938424346993</v>
       </c>
       <c r="H115" t="n">
-        <v>14.99818388012182</v>
+        <v>14.99818388012181</v>
       </c>
       <c r="I115" t="n">
         <v>0</v>
@@ -7492,16 +7492,16 @@
         <v>5</v>
       </c>
       <c r="E116" t="n">
-        <v>0.9693809887714521</v>
+        <v>0.969380988771452</v>
       </c>
       <c r="F116" t="n">
-        <v>0.1593359391369411</v>
+        <v>0.1593359391369412</v>
       </c>
       <c r="G116" t="n">
         <v>0.1262018832180941</v>
       </c>
       <c r="H116" t="n">
-        <v>4.859735350266514</v>
+        <v>4.859735350266516</v>
       </c>
       <c r="I116" t="n">
         <v>0</v>
@@ -7531,13 +7531,13 @@
         <v>0.9852208142476564</v>
       </c>
       <c r="F117" t="n">
-        <v>0.0991407235713474</v>
+        <v>0.09914072357134737</v>
       </c>
       <c r="G117" t="n">
-        <v>0.08504354615413892</v>
+        <v>0.08504354615413887</v>
       </c>
       <c r="H117" t="n">
-        <v>3.607527352467236</v>
+        <v>3.607527352467235</v>
       </c>
       <c r="I117" t="n">
         <v>0</v>
@@ -7567,13 +7567,13 @@
         <v>0.8693668562463999</v>
       </c>
       <c r="F118" t="n">
-        <v>0.4460883181911253</v>
+        <v>0.4460883181911252</v>
       </c>
       <c r="G118" t="n">
-        <v>0.2943752816405159</v>
+        <v>0.2943752816405157</v>
       </c>
       <c r="H118" t="n">
-        <v>19.22302556463011</v>
+        <v>19.22302556463012</v>
       </c>
       <c r="I118" t="n">
         <v>0</v>
@@ -7636,16 +7636,16 @@
         <v>4</v>
       </c>
       <c r="E120" t="n">
-        <v>0.9612734186085253</v>
+        <v>0.9612734186085254</v>
       </c>
       <c r="F120" t="n">
-        <v>0.1722711559237025</v>
+        <v>0.1722711559237023</v>
       </c>
       <c r="G120" t="n">
-        <v>0.1360571628012935</v>
+        <v>0.1360571628012933</v>
       </c>
       <c r="H120" t="n">
-        <v>6.141732887949415</v>
+        <v>6.141732887949407</v>
       </c>
       <c r="I120" t="n">
         <v>0</v>
@@ -7678,10 +7678,10 @@
         <v>0.1656542628144205</v>
       </c>
       <c r="G121" t="n">
-        <v>0.1063554921390487</v>
+        <v>0.1063554921390485</v>
       </c>
       <c r="H121" t="n">
-        <v>5.764421893493064</v>
+        <v>5.764421893493053</v>
       </c>
       <c r="I121" t="n">
         <v>0</v>
@@ -7708,13 +7708,13 @@
         <v>1</v>
       </c>
       <c r="E122" t="n">
-        <v>0.9866601513592257</v>
+        <v>0.9866601513592256</v>
       </c>
       <c r="F122" t="n">
-        <v>0.1155040492915211</v>
+        <v>0.1155040492915212</v>
       </c>
       <c r="G122" t="n">
-        <v>0.07457030718433484</v>
+        <v>0.0745703071843349</v>
       </c>
       <c r="H122" t="n">
         <v>4.780084397090167</v>
@@ -7780,16 +7780,16 @@
         <v>3</v>
       </c>
       <c r="E124" t="n">
-        <v>0.9716585955882552</v>
+        <v>0.9716585955882551</v>
       </c>
       <c r="F124" t="n">
-        <v>0.1762942197453881</v>
+        <v>0.1762942197453884</v>
       </c>
       <c r="G124" t="n">
-        <v>0.09899644177433484</v>
+        <v>0.09899644177433498</v>
       </c>
       <c r="H124" t="n">
-        <v>3.037153665191175</v>
+        <v>3.037153665191179</v>
       </c>
       <c r="I124" t="n">
         <v>0</v>
@@ -7816,16 +7816,16 @@
         <v>4</v>
       </c>
       <c r="E125" t="n">
-        <v>0.6428603554542116</v>
+        <v>0.6428603554542121</v>
       </c>
       <c r="F125" t="n">
-        <v>0.590847737364413</v>
+        <v>0.5908477373644128</v>
       </c>
       <c r="G125" t="n">
-        <v>0.3167908385028481</v>
+        <v>0.316790838502848</v>
       </c>
       <c r="H125" t="n">
-        <v>25.77714418718726</v>
+        <v>25.77714418718725</v>
       </c>
       <c r="I125" t="n">
         <v>0</v>
@@ -7855,13 +7855,13 @@
         <v>0.9610906515533014</v>
       </c>
       <c r="F126" t="n">
-        <v>0.1539540620631567</v>
+        <v>0.1539540620631566</v>
       </c>
       <c r="G126" t="n">
         <v>0.1078454326928352</v>
       </c>
       <c r="H126" t="n">
-        <v>5.359268492903667</v>
+        <v>5.359268492903664</v>
       </c>
       <c r="I126" t="n">
         <v>0</v>
@@ -7891,13 +7891,13 @@
         <v>0.9874849148732718</v>
       </c>
       <c r="F127" t="n">
-        <v>0.09363611803677883</v>
+        <v>0.09363611803677868</v>
       </c>
       <c r="G127" t="n">
-        <v>0.07125241581807566</v>
+        <v>0.07125241581807543</v>
       </c>
       <c r="H127" t="n">
-        <v>3.002667572472275</v>
+        <v>3.002667572472267</v>
       </c>
       <c r="I127" t="n">
         <v>0</v>
@@ -7924,13 +7924,13 @@
         <v>2</v>
       </c>
       <c r="E128" t="n">
-        <v>0.9654572853821238</v>
+        <v>0.9654572853821239</v>
       </c>
       <c r="F128" t="n">
-        <v>0.2003378749815371</v>
+        <v>0.2003378749815369</v>
       </c>
       <c r="G128" t="n">
-        <v>0.1177269299819487</v>
+        <v>0.1177269299819486</v>
       </c>
       <c r="H128" t="n">
         <v>6.59629436340076</v>
@@ -7960,7 +7960,7 @@
         <v>3</v>
       </c>
       <c r="E129" t="n">
-        <v>0.8551772652320896</v>
+        <v>0.8551772652320897</v>
       </c>
       <c r="F129" t="n">
         <v>0.3479670726918712</v>
@@ -7999,10 +7999,10 @@
         <v>0.8160604108486245</v>
       </c>
       <c r="F130" t="n">
-        <v>0.3624644979369027</v>
+        <v>0.3624644979369028</v>
       </c>
       <c r="G130" t="n">
-        <v>0.2692417646605758</v>
+        <v>0.2692417646605759</v>
       </c>
       <c r="H130" t="n">
         <v>17.5138657830378</v>
@@ -8035,13 +8035,13 @@
         <v>0.9928322795971171</v>
       </c>
       <c r="F131" t="n">
-        <v>0.07709188972513303</v>
+        <v>0.07709188972513309</v>
       </c>
       <c r="G131" t="n">
-        <v>0.05698884594421753</v>
+        <v>0.05698884594421767</v>
       </c>
       <c r="H131" t="n">
-        <v>2.233367226859502</v>
+        <v>2.233367226859508</v>
       </c>
       <c r="I131" t="n">
         <v>0</v>
@@ -8071,13 +8071,13 @@
         <v>0.989566924239858</v>
       </c>
       <c r="F132" t="n">
-        <v>0.08329770020089544</v>
+        <v>0.08329770020089534</v>
       </c>
       <c r="G132" t="n">
-        <v>0.07457743259315207</v>
+        <v>0.0745774325931519</v>
       </c>
       <c r="H132" t="n">
-        <v>3.322338968162474</v>
+        <v>3.32233896816247</v>
       </c>
       <c r="I132" t="n">
         <v>0</v>
@@ -8107,10 +8107,10 @@
         <v>0.8988013545483511</v>
       </c>
       <c r="F133" t="n">
-        <v>0.392628219815494</v>
+        <v>0.3926282198154939</v>
       </c>
       <c r="G133" t="n">
-        <v>0.2648323846986728</v>
+        <v>0.2648323846986729</v>
       </c>
       <c r="H133" t="n">
         <v>17.43441186490313</v>
@@ -8140,16 +8140,16 @@
         <v>3</v>
       </c>
       <c r="E134" t="n">
-        <v>0.9504587608437873</v>
+        <v>0.9504587608437872</v>
       </c>
       <c r="F134" t="n">
-        <v>0.1762095924989003</v>
+        <v>0.1762095924989004</v>
       </c>
       <c r="G134" t="n">
-        <v>0.1059933417701574</v>
+        <v>0.1059933417701576</v>
       </c>
       <c r="H134" t="n">
-        <v>7.427582934741415</v>
+        <v>7.427582934741424</v>
       </c>
       <c r="I134" t="n">
         <v>0</v>
@@ -8179,13 +8179,13 @@
         <v>0.9450647087479204</v>
       </c>
       <c r="F135" t="n">
-        <v>0.205179375170257</v>
+        <v>0.2051793751702572</v>
       </c>
       <c r="G135" t="n">
-        <v>0.1270922456287762</v>
+        <v>0.1270922456287763</v>
       </c>
       <c r="H135" t="n">
-        <v>7.280415751753069</v>
+        <v>7.280415751753076</v>
       </c>
       <c r="I135" t="n">
         <v>0</v>
@@ -8215,13 +8215,13 @@
         <v>0.976744084626629</v>
       </c>
       <c r="F136" t="n">
-        <v>0.1423323476268569</v>
+        <v>0.1423323476268568</v>
       </c>
       <c r="G136" t="n">
-        <v>0.09892010191190569</v>
+        <v>0.09892010191190548</v>
       </c>
       <c r="H136" t="n">
-        <v>5.431636557972968</v>
+        <v>5.431636557972957</v>
       </c>
       <c r="I136" t="n">
         <v>0</v>
@@ -10948,16 +10948,16 @@
         <v>1</v>
       </c>
       <c r="E212" t="n">
-        <v>0.9523698612024207</v>
+        <v>0.9523698612024208</v>
       </c>
       <c r="F212" t="n">
-        <v>0.01993544697724106</v>
+        <v>0.01993544697724105</v>
       </c>
       <c r="G212" t="n">
-        <v>0.01437423855498198</v>
+        <v>0.01437423855498197</v>
       </c>
       <c r="H212" t="n">
-        <v>15.43430499284793</v>
+        <v>15.43430499284792</v>
       </c>
       <c r="I212" t="n">
         <v>0</v>
@@ -10987,13 +10987,13 @@
         <v>0.9710868763549413</v>
       </c>
       <c r="F213" t="n">
-        <v>0.01665611840197983</v>
+        <v>0.01665611840197984</v>
       </c>
       <c r="G213" t="n">
         <v>0.01317581672774595</v>
       </c>
       <c r="H213" t="n">
-        <v>7.051883197478862</v>
+        <v>7.051883197478863</v>
       </c>
       <c r="I213" t="n">
         <v>0</v>
@@ -11026,10 +11026,10 @@
         <v>0.02120989239307004</v>
       </c>
       <c r="G214" t="n">
-        <v>0.01629545983662409</v>
+        <v>0.01629545983662408</v>
       </c>
       <c r="H214" t="n">
-        <v>9.966185130305693</v>
+        <v>9.966185130305687</v>
       </c>
       <c r="I214" t="n">
         <v>0</v>
@@ -11062,7 +11062,7 @@
         <v>0.02136462979580206</v>
       </c>
       <c r="G215" t="n">
-        <v>0.01598473292993874</v>
+        <v>0.01598473292993872</v>
       </c>
       <c r="H215" t="n">
         <v>13.11668690628473</v>
@@ -11095,10 +11095,10 @@
         <v>0.9856982582102578</v>
       </c>
       <c r="F216" t="n">
-        <v>0.008965522121549807</v>
+        <v>0.008965522121549808</v>
       </c>
       <c r="G216" t="n">
-        <v>0.007055855716542111</v>
+        <v>0.007055855716542104</v>
       </c>
       <c r="H216" t="n">
         <v>5.020688752422924</v>
@@ -11131,13 +11131,13 @@
         <v>0.9668639782792819</v>
       </c>
       <c r="F217" t="n">
-        <v>0.01735457777685738</v>
+        <v>0.01735457777685739</v>
       </c>
       <c r="G217" t="n">
-        <v>0.01313413779906128</v>
+        <v>0.0131341377990613</v>
       </c>
       <c r="H217" t="n">
-        <v>9.973236290837727</v>
+        <v>9.973236290837731</v>
       </c>
       <c r="I217" t="n">
         <v>0</v>
@@ -11164,16 +11164,16 @@
         <v>2</v>
       </c>
       <c r="E218" t="n">
-        <v>0.9582557174381657</v>
+        <v>0.9582557174381655</v>
       </c>
       <c r="F218" t="n">
-        <v>0.01999340753255932</v>
+        <v>0.01999340753255936</v>
       </c>
       <c r="G218" t="n">
-        <v>0.01685530366627239</v>
+        <v>0.01685530366627242</v>
       </c>
       <c r="H218" t="n">
-        <v>9.573707620589806</v>
+        <v>9.573707620589818</v>
       </c>
       <c r="I218" t="n">
         <v>0</v>
@@ -11203,7 +11203,7 @@
         <v>0.9033181981904492</v>
       </c>
       <c r="F219" t="n">
-        <v>0.02784016292516088</v>
+        <v>0.02784016292516089</v>
       </c>
       <c r="G219" t="n">
         <v>0.02300961239288796</v>
@@ -11239,13 +11239,13 @@
         <v>0.9836034652871317</v>
       </c>
       <c r="F220" t="n">
-        <v>0.01349575922051203</v>
+        <v>0.013495759220512</v>
       </c>
       <c r="G220" t="n">
-        <v>0.01077927886044781</v>
+        <v>0.01077927886044778</v>
       </c>
       <c r="H220" t="n">
-        <v>11.80817783286247</v>
+        <v>11.80817783286246</v>
       </c>
       <c r="I220" t="n">
         <v>0</v>
@@ -11272,16 +11272,16 @@
         <v>5</v>
       </c>
       <c r="E221" t="n">
-        <v>0.9115028567858942</v>
+        <v>0.9115028567858939</v>
       </c>
       <c r="F221" t="n">
-        <v>0.02092798635659659</v>
+        <v>0.02092798635659661</v>
       </c>
       <c r="G221" t="n">
-        <v>0.01540176534418788</v>
+        <v>0.01540176534418789</v>
       </c>
       <c r="H221" t="n">
-        <v>10.23374506384253</v>
+        <v>10.23374506384254</v>
       </c>
       <c r="I221" t="n">
         <v>0</v>
@@ -11311,13 +11311,13 @@
         <v>0.9749939272362897</v>
       </c>
       <c r="F222" t="n">
-        <v>0.01296871070605219</v>
+        <v>0.01296871070605218</v>
       </c>
       <c r="G222" t="n">
-        <v>0.01164676159030183</v>
+        <v>0.01164676159030181</v>
       </c>
       <c r="H222" t="n">
-        <v>6.81509156077199</v>
+        <v>6.815091560771984</v>
       </c>
       <c r="I222" t="n">
         <v>0</v>
@@ -11347,13 +11347,13 @@
         <v>0.965098727627073</v>
       </c>
       <c r="F223" t="n">
-        <v>0.02120188583139749</v>
+        <v>0.0212018858313975</v>
       </c>
       <c r="G223" t="n">
-        <v>0.01727509974682844</v>
+        <v>0.01727509974682847</v>
       </c>
       <c r="H223" t="n">
-        <v>7.773378213146322</v>
+        <v>7.773378213146333</v>
       </c>
       <c r="I223" t="n">
         <v>0</v>
@@ -11383,13 +11383,13 @@
         <v>0.9540305130685156</v>
       </c>
       <c r="F224" t="n">
-        <v>0.01983890233977028</v>
+        <v>0.01983890233977029</v>
       </c>
       <c r="G224" t="n">
-        <v>0.01620243577423805</v>
+        <v>0.01620243577423806</v>
       </c>
       <c r="H224" t="n">
-        <v>11.24973492360362</v>
+        <v>11.24973492360363</v>
       </c>
       <c r="I224" t="n">
         <v>0</v>
@@ -11452,16 +11452,16 @@
         <v>5</v>
       </c>
       <c r="E226" t="n">
-        <v>0.9561498637310073</v>
+        <v>0.9561498637310074</v>
       </c>
       <c r="F226" t="n">
-        <v>0.01906715540839439</v>
+        <v>0.01906715540839437</v>
       </c>
       <c r="G226" t="n">
-        <v>0.01486580996495148</v>
+        <v>0.01486580996495146</v>
       </c>
       <c r="H226" t="n">
-        <v>18.6523417118313</v>
+        <v>18.65234171183129</v>
       </c>
       <c r="I226" t="n">
         <v>0</v>
@@ -11494,10 +11494,10 @@
         <v>0.02088864802597445</v>
       </c>
       <c r="G227" t="n">
-        <v>0.01507835227550757</v>
+        <v>0.01507835227550756</v>
       </c>
       <c r="H227" t="n">
-        <v>18.35115454617269</v>
+        <v>18.35115454617268</v>
       </c>
       <c r="I227" t="n">
         <v>0</v>
@@ -11527,13 +11527,13 @@
         <v>0.9847593783475063</v>
       </c>
       <c r="F228" t="n">
-        <v>0.01209282125643309</v>
+        <v>0.0120928212564331</v>
       </c>
       <c r="G228" t="n">
-        <v>0.008614806604091947</v>
+        <v>0.008614806604091942</v>
       </c>
       <c r="H228" t="n">
-        <v>4.812061238341384</v>
+        <v>4.812061238341381</v>
       </c>
       <c r="I228" t="n">
         <v>0</v>
@@ -11560,10 +11560,10 @@
         <v>3</v>
       </c>
       <c r="E229" t="n">
-        <v>0.93955379398399</v>
+        <v>0.9395537939839899</v>
       </c>
       <c r="F229" t="n">
-        <v>0.02075688041959624</v>
+        <v>0.02075688041959626</v>
       </c>
       <c r="G229" t="n">
         <v>0.01418382090054971</v>
@@ -11596,16 +11596,16 @@
         <v>4</v>
       </c>
       <c r="E230" t="n">
-        <v>0.9517068660571898</v>
+        <v>0.9517068660571899</v>
       </c>
       <c r="F230" t="n">
-        <v>0.02628582010908896</v>
+        <v>0.02628582010908895</v>
       </c>
       <c r="G230" t="n">
-        <v>0.01994340896636357</v>
+        <v>0.01994340896636354</v>
       </c>
       <c r="H230" t="n">
-        <v>20.72434986096759</v>
+        <v>20.72434986096757</v>
       </c>
       <c r="I230" t="n">
         <v>0</v>
@@ -11635,13 +11635,13 @@
         <v>0.9890691418825734</v>
       </c>
       <c r="F231" t="n">
-        <v>0.007838053953929431</v>
+        <v>0.00783805395392944</v>
       </c>
       <c r="G231" t="n">
-        <v>0.006775579531163867</v>
+        <v>0.00677557953116387</v>
       </c>
       <c r="H231" t="n">
-        <v>4.84033840253295</v>
+        <v>4.840338402532952</v>
       </c>
       <c r="I231" t="n">
         <v>0</v>
@@ -11677,7 +11677,7 @@
         <v>0.0140295889844973</v>
       </c>
       <c r="H232" t="n">
-        <v>10.13173184813296</v>
+        <v>10.13173184813297</v>
       </c>
       <c r="I232" t="n">
         <v>0</v>
@@ -11707,10 +11707,10 @@
         <v>0.9624537312880868</v>
       </c>
       <c r="F233" t="n">
-        <v>0.01896145718404662</v>
+        <v>0.01896145718404661</v>
       </c>
       <c r="G233" t="n">
-        <v>0.01325727397321584</v>
+        <v>0.01325727397321583</v>
       </c>
       <c r="H233" t="n">
         <v>9.694311900741608</v>
@@ -11746,7 +11746,7 @@
         <v>0.02289330852799992</v>
       </c>
       <c r="G234" t="n">
-        <v>0.01674607251196245</v>
+        <v>0.01674607251196243</v>
       </c>
       <c r="H234" t="n">
         <v>22.71837783161589</v>
@@ -11779,10 +11779,10 @@
         <v>0.9918525678848983</v>
       </c>
       <c r="F235" t="n">
-        <v>0.00951331024923999</v>
+        <v>0.009513310249239982</v>
       </c>
       <c r="G235" t="n">
-        <v>0.007683528576124644</v>
+        <v>0.00768352857612464</v>
       </c>
       <c r="H235" t="n">
         <v>10.91036870335591</v>
@@ -11815,13 +11815,13 @@
         <v>0.9750669735871933</v>
       </c>
       <c r="F236" t="n">
-        <v>0.01110836947478371</v>
+        <v>0.0111083694747837</v>
       </c>
       <c r="G236" t="n">
-        <v>0.009379296719200294</v>
+        <v>0.00937929671920028</v>
       </c>
       <c r="H236" t="n">
-        <v>6.601208766818008</v>
+        <v>6.601208766818003</v>
       </c>
       <c r="I236" t="n">
         <v>0</v>
@@ -11854,10 +11854,10 @@
         <v>0.007890571770025601</v>
       </c>
       <c r="G237" t="n">
-        <v>0.006256267178279891</v>
+        <v>0.006256267178279895</v>
       </c>
       <c r="H237" t="n">
-        <v>5.079349782303521</v>
+        <v>5.079349782303524</v>
       </c>
       <c r="I237" t="n">
         <v>0</v>
@@ -11884,16 +11884,16 @@
         <v>2</v>
       </c>
       <c r="E238" t="n">
-        <v>0.9656561269897267</v>
+        <v>0.9656561269897266</v>
       </c>
       <c r="F238" t="n">
-        <v>0.02103189942862632</v>
+        <v>0.02103189942862637</v>
       </c>
       <c r="G238" t="n">
-        <v>0.01593030704531249</v>
+        <v>0.0159303070453125</v>
       </c>
       <c r="H238" t="n">
-        <v>6.255185135725047</v>
+        <v>6.255185135725048</v>
       </c>
       <c r="I238" t="n">
         <v>0</v>
@@ -11920,16 +11920,16 @@
         <v>3</v>
       </c>
       <c r="E239" t="n">
-        <v>0.957994245886501</v>
+        <v>0.9579942458865011</v>
       </c>
       <c r="F239" t="n">
-        <v>0.01896431691126525</v>
+        <v>0.01896431691126523</v>
       </c>
       <c r="G239" t="n">
         <v>0.01327869421054759</v>
       </c>
       <c r="H239" t="n">
-        <v>11.16703569446049</v>
+        <v>11.16703569446048</v>
       </c>
       <c r="I239" t="n">
         <v>0</v>
@@ -11959,10 +11959,10 @@
         <v>0.9722424397053584</v>
       </c>
       <c r="F240" t="n">
-        <v>0.01606690160332386</v>
+        <v>0.01606690160332387</v>
       </c>
       <c r="G240" t="n">
-        <v>0.01243741149790238</v>
+        <v>0.01243741149790239</v>
       </c>
       <c r="H240" t="n">
         <v>13.63173403867667</v>
@@ -12001,7 +12001,7 @@
         <v>0.01470857329186766</v>
       </c>
       <c r="H241" t="n">
-        <v>19.89224191135751</v>
+        <v>19.8922419113575</v>
       </c>
       <c r="I241" t="n">
         <v>0</v>
@@ -14791,7 +14791,7 @@
         <v>0.934595006210568</v>
       </c>
       <c r="D2" t="n">
-        <v>0.04789873615059224</v>
+        <v>0.04789873615059226</v>
       </c>
       <c r="E2" t="n">
         <v>0.05773522570429511</v>
@@ -14863,7 +14863,7 @@
         <v>0.9644925796153505</v>
       </c>
       <c r="D4" t="n">
-        <v>0.01851395006701762</v>
+        <v>0.01851395006701763</v>
       </c>
       <c r="E4" t="n">
         <v>0.01698790673322198</v>
@@ -14878,7 +14878,7 @@
         <v>0.006280417543781659</v>
       </c>
       <c r="I4" t="n">
-        <v>3.951480282121468</v>
+        <v>3.951480282121467</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -14995,10 +14995,10 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>0.05758305566816652</v>
+        <v>0.05758305566816653</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.03424972266816652</v>
+        <v>-0.03424972266816653</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -15070,10 +15070,10 @@
         </is>
       </c>
       <c r="M3" t="n">
-        <v>0.1652224885391159</v>
+        <v>0.165222488539116</v>
       </c>
       <c r="N3" t="n">
-        <v>-0.009709141539115951</v>
+        <v>-0.009709141539115979</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -15101,10 +15101,10 @@
         <v>0.180976271</v>
       </c>
       <c r="G4" t="n">
-        <v>0.964594166433333</v>
+        <v>0.9645941664333332</v>
       </c>
       <c r="H4" t="n">
-        <v>0.0220725005666671</v>
+        <v>0.02207250056666687</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -15126,7 +15126,7 @@
         <v>0.1790178136855087</v>
       </c>
       <c r="N4" t="n">
-        <v>0.001958457314491319</v>
+        <v>0.001958457314491291</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -15154,10 +15154,10 @@
         <v>0.12191595</v>
       </c>
       <c r="G5" t="n">
-        <v>0.5456977778628334</v>
+        <v>0.5456977778628335</v>
       </c>
       <c r="H5" t="n">
-        <v>0.06096888913716669</v>
+        <v>0.06096888913716658</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -15176,10 +15176,10 @@
         </is>
       </c>
       <c r="M5" t="n">
-        <v>0.09907593066991689</v>
+        <v>0.09907593066991688</v>
       </c>
       <c r="N5" t="n">
-        <v>0.0228400193300831</v>
+        <v>0.02284001933008312</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -15260,10 +15260,10 @@
         <v>0.269507547</v>
       </c>
       <c r="G7" t="n">
-        <v>0.9741127775504163</v>
+        <v>0.9741127775504161</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0125538894495838</v>
+        <v>0.01255388944958391</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -15282,10 +15282,10 @@
         </is>
       </c>
       <c r="M7" t="n">
-        <v>0.2568515779369683</v>
+        <v>0.2568515779369682</v>
       </c>
       <c r="N7" t="n">
-        <v>0.01265596906303174</v>
+        <v>0.01265596906303179</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -15366,10 +15366,10 @@
         <v>0.249815332</v>
       </c>
       <c r="G9" t="n">
-        <v>0.8448402779424994</v>
+        <v>0.8448402779424993</v>
       </c>
       <c r="H9" t="n">
-        <v>0.0151597220575006</v>
+        <v>0.01515972205750071</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -15525,10 +15525,10 @@
         <v>0.260389238</v>
       </c>
       <c r="G12" t="n">
-        <v>0.788905555594334</v>
+        <v>0.7889055555943338</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.002238888594333965</v>
+        <v>-0.002238888594333854</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -15578,10 +15578,10 @@
         <v>0.328983913</v>
       </c>
       <c r="G13" t="n">
-        <v>0.950816666695834</v>
+        <v>0.9508166666958339</v>
       </c>
       <c r="H13" t="n">
-        <v>0.005850000304166048</v>
+        <v>0.005850000304166159</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -15600,10 +15600,10 @@
         </is>
       </c>
       <c r="M13" t="n">
-        <v>0.3114627807294167</v>
+        <v>0.3114627807294168</v>
       </c>
       <c r="N13" t="n">
-        <v>0.01752113227058327</v>
+        <v>0.01752113227058322</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -15684,10 +15684,10 @@
         <v>0.281931145</v>
       </c>
       <c r="G15" t="n">
-        <v>0.7900263887904175</v>
+        <v>0.7900263887904174</v>
       </c>
       <c r="H15" t="n">
-        <v>-2.638879041749753e-05</v>
+        <v>-2.638879041738651e-05</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -15709,7 +15709,7 @@
         <v>0.2814747560275001</v>
       </c>
       <c r="N15" t="n">
-        <v>0.0004563889724999437</v>
+        <v>0.0004563889724998882</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -15737,10 +15737,10 @@
         <v>0.330783285</v>
       </c>
       <c r="G16" t="n">
-        <v>0.9199805557770828</v>
+        <v>0.9199805557770833</v>
       </c>
       <c r="H16" t="n">
-        <v>-0.01664722277708286</v>
+        <v>-0.0166472227770833</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -15759,10 +15759,10 @@
         </is>
       </c>
       <c r="M16" t="n">
-        <v>0.3326050503066665</v>
+        <v>0.3326050503066666</v>
       </c>
       <c r="N16" t="n">
-        <v>-0.001821765306666501</v>
+        <v>-0.001821765306666612</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -15815,7 +15815,7 @@
         <v>0.1594327603488888</v>
       </c>
       <c r="N17" t="n">
-        <v>-0.008124599348888817</v>
+        <v>-0.008124599348888789</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -15843,10 +15843,10 @@
         <v>0.255832691</v>
       </c>
       <c r="G18" t="n">
-        <v>0.7193327776292507</v>
+        <v>0.7193327776292506</v>
       </c>
       <c r="H18" t="n">
-        <v>-0.02933277762925079</v>
+        <v>-0.02933277762925068</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -15868,7 +15868,7 @@
         <v>0.2640848844708892</v>
       </c>
       <c r="N18" t="n">
-        <v>-0.008252193470889235</v>
+        <v>-0.00825219347088918</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -15981,10 +15981,10 @@
         <v>0.486666667</v>
       </c>
       <c r="E2" t="n">
-        <v>0.4060052778498331</v>
+        <v>0.4060052778498329</v>
       </c>
       <c r="F2" t="n">
-        <v>0.08066138915016691</v>
+        <v>0.08066138915016713</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -16034,10 +16034,10 @@
         <v>0.67</v>
       </c>
       <c r="E3" t="n">
-        <v>0.5842780556308335</v>
+        <v>0.5842780556308333</v>
       </c>
       <c r="F3" t="n">
-        <v>0.08572194436916658</v>
+        <v>0.08572194436916669</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -16087,10 +16087,10 @@
         <v>0.76</v>
       </c>
       <c r="E4" t="n">
-        <v>0.7329769445350844</v>
+        <v>0.7329769445350842</v>
       </c>
       <c r="F4" t="n">
-        <v>0.02702305546491557</v>
+        <v>0.02702305546491579</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -16115,10 +16115,10 @@
         <v>0.09732962000000001</v>
       </c>
       <c r="M4" t="n">
-        <v>0.1296423415908241</v>
+        <v>0.1296423415908242</v>
       </c>
       <c r="N4" t="n">
-        <v>-0.03231272159082413</v>
+        <v>-0.03231272159082416</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -16193,10 +16193,10 @@
         <v>0.846666667</v>
       </c>
       <c r="E6" t="n">
-        <v>0.8332783333813351</v>
+        <v>0.8332783333813348</v>
       </c>
       <c r="F6" t="n">
-        <v>0.01338833361866498</v>
+        <v>0.0133883336186652</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -16221,10 +16221,10 @@
         <v>0.129812368</v>
       </c>
       <c r="M6" t="n">
-        <v>0.1424692913957825</v>
+        <v>0.1424692913957826</v>
       </c>
       <c r="N6" t="n">
-        <v>-0.01265692339578253</v>
+        <v>-0.01265692339578256</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -16246,10 +16246,10 @@
         <v>0.87</v>
       </c>
       <c r="E7" t="n">
-        <v>0.8638866666309175</v>
+        <v>0.8638866666309174</v>
       </c>
       <c r="F7" t="n">
-        <v>0.006113333369082485</v>
+        <v>0.006113333369082596</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -16352,10 +16352,10 @@
         <v>0.933333333</v>
       </c>
       <c r="E9" t="n">
-        <v>0.9238166665312499</v>
+        <v>0.9238166665312498</v>
       </c>
       <c r="F9" t="n">
-        <v>0.009516666468750046</v>
+        <v>0.009516666468750157</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -16380,10 +16380,10 @@
         <v>0.162426774</v>
       </c>
       <c r="M9" t="n">
-        <v>0.1662017848620326</v>
+        <v>0.1662017848620325</v>
       </c>
       <c r="N9" t="n">
-        <v>-0.00377501086203258</v>
+        <v>-0.003775010862032552</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -16433,10 +16433,10 @@
         <v>0.167631151</v>
       </c>
       <c r="M10" t="n">
-        <v>0.1663562588295326</v>
+        <v>0.1663562588295325</v>
       </c>
       <c r="N10" t="n">
-        <v>0.001274892170467418</v>
+        <v>0.001274892170467473</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -16458,10 +16458,10 @@
         <v>0.963333333</v>
       </c>
       <c r="E11" t="n">
-        <v>0.9554972219720006</v>
+        <v>0.9554972219720007</v>
       </c>
       <c r="F11" t="n">
-        <v>0.007836111027999415</v>
+        <v>0.007836111027999304</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -16511,10 +16511,10 @@
         <v>0.993333333</v>
       </c>
       <c r="E12" t="n">
-        <v>0.9768580552704157</v>
+        <v>0.9768580552704158</v>
       </c>
       <c r="F12" t="n">
-        <v>0.01647527772958435</v>
+        <v>0.01647527772958424</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -16539,10 +16539,10 @@
         <v>0.185595806</v>
       </c>
       <c r="M12" t="n">
-        <v>0.1822463884571754</v>
+        <v>0.1822463884571755</v>
       </c>
       <c r="N12" t="n">
-        <v>0.003349417542824584</v>
+        <v>0.003349417542824501</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -16617,10 +16617,10 @@
         <v>0.413333333</v>
       </c>
       <c r="E14" t="n">
-        <v>0.3661488889406668</v>
+        <v>0.3661488889406667</v>
       </c>
       <c r="F14" t="n">
-        <v>0.0471844440593332</v>
+        <v>0.04718444405933331</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -16670,10 +16670,10 @@
         <v>0.706666667</v>
       </c>
       <c r="E15" t="n">
-        <v>0.7100533335465837</v>
+        <v>0.7100533335465836</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.003386666546583705</v>
+        <v>-0.003386666546583594</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -16698,10 +16698,10 @@
         <v>0.160936952</v>
       </c>
       <c r="M15" t="n">
-        <v>0.1519708527161109</v>
+        <v>0.151970852716111</v>
       </c>
       <c r="N15" t="n">
-        <v>0.008966099283889056</v>
+        <v>0.008966099283889029</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -16723,10 +16723,10 @@
         <v>0.766666667</v>
       </c>
       <c r="E16" t="n">
-        <v>0.7684483334601666</v>
+        <v>0.7684483334601667</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.001781666460166642</v>
+        <v>-0.001781666460166753</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -16754,7 +16754,7 @@
         <v>0.1782121026726945</v>
       </c>
       <c r="N16" t="n">
-        <v>0.004422472327305499</v>
+        <v>0.004422472327305527</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -16776,10 +16776,10 @@
         <v>0.8100000000000001</v>
       </c>
       <c r="E17" t="n">
-        <v>0.806574166772</v>
+        <v>0.8065741667720003</v>
       </c>
       <c r="F17" t="n">
-        <v>0.003425833228000053</v>
+        <v>0.003425833227999719</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -16829,10 +16829,10 @@
         <v>0.85</v>
       </c>
       <c r="E18" t="n">
-        <v>0.8438127777835845</v>
+        <v>0.8438127777835844</v>
       </c>
       <c r="F18" t="n">
-        <v>0.006187222216415433</v>
+        <v>0.006187222216415544</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -16913,7 +16913,7 @@
         <v>0.2421940702550513</v>
       </c>
       <c r="N19" t="n">
-        <v>-0.006028807255051283</v>
+        <v>-0.006028807255051311</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -16935,10 +16935,10 @@
         <v>0.916666667</v>
       </c>
       <c r="E20" t="n">
-        <v>0.9170002778154166</v>
+        <v>0.9170002778154165</v>
       </c>
       <c r="F20" t="n">
-        <v>-0.0003336108154166073</v>
+        <v>-0.0003336108154164963</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -16963,10 +16963,10 @@
         <v>0.241661312</v>
       </c>
       <c r="M20" t="n">
-        <v>0.2442694872080514</v>
+        <v>0.2442694872080515</v>
       </c>
       <c r="N20" t="n">
-        <v>-0.0026081752080514</v>
+        <v>-0.002608175208051483</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -16988,10 +16988,10 @@
         <v>0.946666667</v>
       </c>
       <c r="E21" t="n">
-        <v>0.9427055556212496</v>
+        <v>0.9427055556212492</v>
       </c>
       <c r="F21" t="n">
-        <v>0.003961111378750437</v>
+        <v>0.00396111137875077</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -17019,7 +17019,7 @@
         <v>0.2493404244808849</v>
       </c>
       <c r="N21" t="n">
-        <v>0.003466115519115159</v>
+        <v>0.003466115519115132</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -17041,10 +17041,10 @@
         <v>0.95</v>
       </c>
       <c r="E22" t="n">
-        <v>0.9483244444164167</v>
+        <v>0.9483244444164168</v>
       </c>
       <c r="F22" t="n">
-        <v>0.001675555583583233</v>
+        <v>0.001675555583583122</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -17072,7 +17072,7 @@
         <v>0.2550088921035515</v>
       </c>
       <c r="N22" t="n">
-        <v>0.001516359896448438</v>
+        <v>0.001516359896448494</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -17094,10 +17094,10 @@
         <v>0.973333333</v>
       </c>
       <c r="E23" t="n">
-        <v>0.9620930554149999</v>
+        <v>0.962093055415</v>
       </c>
       <c r="F23" t="n">
-        <v>0.01124027758500012</v>
+        <v>0.01124027758500001</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -17125,7 +17125,7 @@
         <v>0.2560676946468849</v>
       </c>
       <c r="N23" t="n">
-        <v>0.007698287353115063</v>
+        <v>0.007698287353115119</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -17147,10 +17147,10 @@
         <v>0.306666667</v>
       </c>
       <c r="E24" t="n">
-        <v>0.3129150000880003</v>
+        <v>0.3129150000880004</v>
       </c>
       <c r="F24" t="n">
-        <v>-0.006248333088000324</v>
+        <v>-0.00624833308800038</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -17175,10 +17175,10 @@
         <v>0.047106137</v>
       </c>
       <c r="M24" t="n">
-        <v>0.04073194331166664</v>
+        <v>0.04073194331166665</v>
       </c>
       <c r="N24" t="n">
-        <v>0.006374193688333363</v>
+        <v>0.006374193688333349</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -17200,10 +17200,10 @@
         <v>0.506666667</v>
       </c>
       <c r="E25" t="n">
-        <v>0.4900313889781671</v>
+        <v>0.4900313889781672</v>
       </c>
       <c r="F25" t="n">
-        <v>0.01663527802183284</v>
+        <v>0.01663527802183279</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -17334,10 +17334,10 @@
         <v>0.17723433</v>
       </c>
       <c r="M27" t="n">
-        <v>0.1827510993907497</v>
+        <v>0.1827510993907498</v>
       </c>
       <c r="N27" t="n">
-        <v>-0.005516769390749743</v>
+        <v>-0.005516769390749771</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -17359,10 +17359,10 @@
         <v>0.743333333</v>
       </c>
       <c r="E28" t="n">
-        <v>0.7322697220995005</v>
+        <v>0.7322697220995003</v>
       </c>
       <c r="F28" t="n">
-        <v>0.01106361090049957</v>
+        <v>0.01106361090049979</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -17412,10 +17412,10 @@
         <v>0.796666667</v>
       </c>
       <c r="E29" t="n">
-        <v>0.785433889041667</v>
+        <v>0.7854338890416669</v>
       </c>
       <c r="F29" t="n">
-        <v>0.011232777958333</v>
+        <v>0.01123277795833311</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -17440,10 +17440,10 @@
         <v>0.226319718</v>
       </c>
       <c r="M29" t="n">
-        <v>0.2291551210686903</v>
+        <v>0.2291551210686904</v>
       </c>
       <c r="N29" t="n">
-        <v>-0.002835403068690345</v>
+        <v>-0.002835403068690401</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -17465,10 +17465,10 @@
         <v>0.826666667</v>
       </c>
       <c r="E30" t="n">
-        <v>0.8181536113054996</v>
+        <v>0.8181536113054997</v>
       </c>
       <c r="F30" t="n">
-        <v>0.008513055694500449</v>
+        <v>0.008513055694500338</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -17518,10 +17518,10 @@
         <v>0.876666667</v>
       </c>
       <c r="E31" t="n">
-        <v>0.8729725001220829</v>
+        <v>0.8729725001220831</v>
       </c>
       <c r="F31" t="n">
-        <v>0.003694166877917016</v>
+        <v>0.003694166877916905</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -17546,10 +17546,10 @@
         <v>0.256419902</v>
       </c>
       <c r="M31" t="n">
-        <v>0.2613892112053572</v>
+        <v>0.2613892112053573</v>
       </c>
       <c r="N31" t="n">
-        <v>-0.004969309205357209</v>
+        <v>-0.00496930920535732</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
@@ -17571,10 +17571,10 @@
         <v>0.92</v>
       </c>
       <c r="E32" t="n">
-        <v>0.9212605556122502</v>
+        <v>0.9212605556122503</v>
       </c>
       <c r="F32" t="n">
-        <v>-0.001260555612250136</v>
+        <v>-0.001260555612250247</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -17599,10 +17599,10 @@
         <v>0.274482585</v>
       </c>
       <c r="M32" t="n">
-        <v>0.2758118705256905</v>
+        <v>0.2758118705256906</v>
       </c>
       <c r="N32" t="n">
-        <v>-0.001329285525690505</v>
+        <v>-0.00132928552569056</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -17677,10 +17677,10 @@
         <v>0.973333333</v>
       </c>
       <c r="E34" t="n">
-        <v>0.9665527776150007</v>
+        <v>0.9665527776150009</v>
       </c>
       <c r="F34" t="n">
-        <v>0.006780555384999332</v>
+        <v>0.00678055538499911</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -17758,10 +17758,10 @@
         <v>0.049264635</v>
       </c>
       <c r="M35" t="n">
-        <v>0.03937760688499991</v>
+        <v>0.0393776068849999</v>
       </c>
       <c r="N35" t="n">
-        <v>0.009887028115000092</v>
+        <v>0.009887028115000099</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
@@ -17783,10 +17783,10 @@
         <v>0.443333333</v>
       </c>
       <c r="E36" t="n">
-        <v>0.4551786111428331</v>
+        <v>0.455178611142833</v>
       </c>
       <c r="F36" t="n">
-        <v>-0.01184527814283309</v>
+        <v>-0.01184527814283298</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -17814,7 +17814,7 @@
         <v>0.1017626480378335</v>
       </c>
       <c r="N36" t="n">
-        <v>0.01379425096216649</v>
+        <v>0.01379425096216652</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
@@ -17942,10 +17942,10 @@
         <v>0.693333333</v>
       </c>
       <c r="E39" t="n">
-        <v>0.6907869441728329</v>
+        <v>0.690786944172833</v>
       </c>
       <c r="F39" t="n">
-        <v>0.002546388827167068</v>
+        <v>0.002546388827166957</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -17995,10 +17995,10 @@
         <v>0.76</v>
       </c>
       <c r="E40" t="n">
-        <v>0.7484358333613338</v>
+        <v>0.7484358333613339</v>
       </c>
       <c r="F40" t="n">
-        <v>0.01156416663866622</v>
+        <v>0.01156416663866611</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -18076,10 +18076,10 @@
         <v>0.276412389</v>
       </c>
       <c r="M41" t="n">
-        <v>0.2768486706896666</v>
+        <v>0.2768486706896667</v>
       </c>
       <c r="N41" t="n">
-        <v>-0.0004362816896666399</v>
+        <v>-0.000436281689666751</v>
       </c>
       <c r="O41" t="inlineStr">
         <is>
@@ -18235,10 +18235,10 @@
         <v>0.303544856</v>
       </c>
       <c r="M44" t="n">
-        <v>0.3046318060117501</v>
+        <v>0.30463180601175</v>
       </c>
       <c r="N44" t="n">
-        <v>-0.001086950011750076</v>
+        <v>-0.001086950011750021</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
@@ -18260,10 +18260,10 @@
         <v>0.916666667</v>
       </c>
       <c r="E45" t="n">
-        <v>0.9234041669008328</v>
+        <v>0.9234041669008327</v>
       </c>
       <c r="F45" t="n">
-        <v>-0.006737499900832833</v>
+        <v>-0.006737499900832722</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -18313,10 +18313,10 @@
         <v>0.043333333</v>
       </c>
       <c r="E46" t="n">
-        <v>0.03234722232833328</v>
+        <v>0.03234722232833327</v>
       </c>
       <c r="F46" t="n">
-        <v>0.01098611067166672</v>
+        <v>0.01098611067166673</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -18419,10 +18419,10 @@
         <v>0.39</v>
       </c>
       <c r="E48" t="n">
-        <v>0.4047691667609161</v>
+        <v>0.4047691667609163</v>
       </c>
       <c r="F48" t="n">
-        <v>-0.01476916676091611</v>
+        <v>-0.01476916676091627</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -18450,7 +18450,7 @@
         <v>0.1024258160703335</v>
       </c>
       <c r="N48" t="n">
-        <v>0.007106461929666505</v>
+        <v>0.007106461929666491</v>
       </c>
       <c r="O48" t="inlineStr">
         <is>
@@ -18556,7 +18556,7 @@
         <v>0.2157175850681664</v>
       </c>
       <c r="N50" t="n">
-        <v>0.003971557931833597</v>
+        <v>0.003971557931833652</v>
       </c>
       <c r="O50" t="inlineStr">
         <is>
@@ -18578,10 +18578,10 @@
         <v>0.71</v>
       </c>
       <c r="E51" t="n">
-        <v>0.7068633332545839</v>
+        <v>0.7068633332545836</v>
       </c>
       <c r="F51" t="n">
-        <v>0.003136666745416017</v>
+        <v>0.00313666674541635</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -18606,10 +18606,10 @@
         <v>0.249950795</v>
       </c>
       <c r="M51" t="n">
-        <v>0.2440511966975004</v>
+        <v>0.2440511966975003</v>
       </c>
       <c r="N51" t="n">
-        <v>0.005899598302499642</v>
+        <v>0.005899598302499726</v>
       </c>
       <c r="O51" t="inlineStr">
         <is>
@@ -18631,10 +18631,10 @@
         <v>0.753333333</v>
       </c>
       <c r="E52" t="n">
-        <v>0.7487691665209174</v>
+        <v>0.7487691665209175</v>
       </c>
       <c r="F52" t="n">
-        <v>0.004564166479082643</v>
+        <v>0.004564166479082532</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -18684,10 +18684,10 @@
         <v>0.83</v>
       </c>
       <c r="E53" t="n">
-        <v>0.8248224999687501</v>
+        <v>0.82482249996875</v>
       </c>
       <c r="F53" t="n">
-        <v>0.005177500031249838</v>
+        <v>0.005177500031249949</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -18712,10 +18712,10 @@
         <v>0.298662612</v>
       </c>
       <c r="M53" t="n">
-        <v>0.2972756659563331</v>
+        <v>0.297275665956333</v>
       </c>
       <c r="N53" t="n">
-        <v>0.001386946043666848</v>
+        <v>0.001386946043666959</v>
       </c>
       <c r="O53" t="inlineStr">
         <is>
@@ -18790,10 +18790,10 @@
         <v>0.896666667</v>
       </c>
       <c r="E55" t="n">
-        <v>0.8880688889955834</v>
+        <v>0.8880688889955836</v>
       </c>
       <c r="F55" t="n">
-        <v>0.008597778004416523</v>
+        <v>0.008597778004416412</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -18843,10 +18843,10 @@
         <v>0.946666667</v>
       </c>
       <c r="E56" t="n">
-        <v>0.94845416675375</v>
+        <v>0.9484541667537502</v>
       </c>
       <c r="F56" t="n">
-        <v>-0.001787499753750033</v>
+        <v>-0.001787499753750144</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -18896,10 +18896,10 @@
         <v>0.026666667</v>
       </c>
       <c r="E57" t="n">
-        <v>0.03234722232833328</v>
+        <v>0.03234722232833327</v>
       </c>
       <c r="F57" t="n">
-        <v>-0.005680555328333278</v>
+        <v>-0.005680555328333271</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -19002,10 +19002,10 @@
         <v>0.316666667</v>
       </c>
       <c r="E59" t="n">
-        <v>0.4050775000983327</v>
+        <v>0.4050775000983329</v>
       </c>
       <c r="F59" t="n">
-        <v>-0.0884108330983327</v>
+        <v>-0.08841083309833292</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -19033,7 +19033,7 @@
         <v>0.1027749715578335</v>
       </c>
       <c r="N59" t="n">
-        <v>-0.005448884557833489</v>
+        <v>-0.005448884557833503</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
@@ -19086,7 +19086,7 @@
         <v>0.188934841841722</v>
       </c>
       <c r="N60" t="n">
-        <v>-0.006802556841722013</v>
+        <v>-0.006802556841722041</v>
       </c>
       <c r="O60" t="inlineStr">
         <is>
@@ -19108,10 +19108,10 @@
         <v>0.603333333</v>
       </c>
       <c r="E61" t="n">
-        <v>0.6174272220284174</v>
+        <v>0.6174272220284173</v>
       </c>
       <c r="F61" t="n">
-        <v>-0.01409388902841735</v>
+        <v>-0.01409388902841724</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -19139,7 +19139,7 @@
         <v>0.2156180413545553</v>
       </c>
       <c r="N61" t="n">
-        <v>-0.0009995433545552934</v>
+        <v>-0.0009995433545552657</v>
       </c>
       <c r="O61" t="inlineStr">
         <is>
@@ -19161,10 +19161,10 @@
         <v>0.64</v>
       </c>
       <c r="E62" t="n">
-        <v>0.6659811110308341</v>
+        <v>0.665981111030834</v>
       </c>
       <c r="F62" t="n">
-        <v>-0.02598111103083411</v>
+        <v>-0.025981111030834</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -19192,7 +19192,7 @@
         <v>0.2427565239197225</v>
       </c>
       <c r="N62" t="n">
-        <v>-0.007330649919722543</v>
+        <v>-0.007330649919722515</v>
       </c>
       <c r="O62" t="inlineStr">
         <is>
@@ -19214,10 +19214,10 @@
         <v>0.753333333</v>
       </c>
       <c r="E63" t="n">
-        <v>0.7667716665050003</v>
+        <v>0.7667716665050002</v>
       </c>
       <c r="F63" t="n">
-        <v>-0.01343833350500023</v>
+        <v>-0.01343833350500012</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -19242,10 +19242,10 @@
         <v>0.281800324</v>
       </c>
       <c r="M63" t="n">
-        <v>0.2837971169310557</v>
+        <v>0.2837971169310558</v>
       </c>
       <c r="N63" t="n">
-        <v>-0.001996792931055758</v>
+        <v>-0.001996792931055813</v>
       </c>
       <c r="O63" t="inlineStr">
         <is>
@@ -19404,7 +19404,7 @@
         <v>0.3312894794820556</v>
       </c>
       <c r="N66" t="n">
-        <v>-0.002052134482055545</v>
+        <v>-0.002052134482055601</v>
       </c>
       <c r="O66" t="inlineStr">
         <is>
@@ -19426,10 +19426,10 @@
         <v>0.916666667</v>
       </c>
       <c r="E67" t="n">
-        <v>0.9155430557569997</v>
+        <v>0.9155430557569996</v>
       </c>
       <c r="F67" t="n">
-        <v>0.001123611243000311</v>
+        <v>0.001123611243000422</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -19454,10 +19454,10 @@
         <v>0.35335845</v>
       </c>
       <c r="M67" t="n">
-        <v>0.3451598021112225</v>
+        <v>0.3451598021112224</v>
       </c>
       <c r="N67" t="n">
-        <v>0.008198647888777499</v>
+        <v>0.00819864788877761</v>
       </c>
       <c r="O67" t="inlineStr">
         <is>
@@ -19479,10 +19479,10 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="E68" t="n">
-        <v>0.9426583334295835</v>
+        <v>0.9426583334295836</v>
       </c>
       <c r="F68" t="n">
-        <v>-0.002658333429583548</v>
+        <v>-0.002658333429583659</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -19507,10 +19507,10 @@
         <v>0.367215621</v>
       </c>
       <c r="M68" t="n">
-        <v>0.3522036745882225</v>
+        <v>0.3522036745882224</v>
       </c>
       <c r="N68" t="n">
-        <v>0.01501194641177744</v>
+        <v>0.01501194641177755</v>
       </c>
       <c r="O68" t="inlineStr">
         <is>

</xml_diff>